<commit_message>
Add word "ansvar" to Ordbog.xlsx
</commit_message>
<xml_diff>
--- a/sets/Ordbog.xlsx
+++ b/sets/Ordbog.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -311,9 +311,96 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>7a4cc355-7000-4f85-86c8-08ae732fbcf5</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ansvar</v>
+      </c>
+      <c r="D2" t="str">
+        <v>ansvar</v>
+      </c>
+      <c r="E2" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v>et</v>
+      </c>
+      <c r="G2" t="str">
+        <v>-et</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[ˈanˌsvɑˀ]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001992_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>juridisk eller moralsk forpligtelse til at stå til regnskab, garantere eller sørge for noget eller nogen</v>
+      </c>
+      <c r="K2" t="str">
+        <v>responsibility</v>
+      </c>
+      <c r="L2" t="str" xml:space="preserve">
+        <v xml:space="preserve">andelsselskab med begrænset ansvar
+coorporation with limited liability</v>
+      </c>
+      <c r="M2" t="str">
+        <v>ansvar | Den Danske Ordbog</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://ordnet.dk/ddo/ordbog/ansvar</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://ordnet.dk/ddo/ordbog/ansvar#:~:text=ansvar</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -322,28 +409,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,8 +512,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "vandring" to Ordbog.xlsx
</commit_message>
<xml_diff>
--- a/sets/Ordbog.xlsx
+++ b/sets/Ordbog.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -398,9 +398,95 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>4107c766-90bd-4707-80a2-e4f7c817dcc9</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-30</v>
+      </c>
+      <c r="C3" t="str">
+        <v>vandring</v>
+      </c>
+      <c r="D3" t="str">
+        <v>vandring</v>
+      </c>
+      <c r="E3" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v>en</v>
+      </c>
+      <c r="G3" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[ˈvɑndʁεŋ]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/12005/12005739_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v>det at vandre en længere strækning (i naturen); det at rejse rundt til fods; vandretur</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Walking</v>
+      </c>
+      <c r="L3" t="str">
+        <v>SPOR skal opleves i naturen. Med høretelefoner i ørerne kan du opleve de stedsspecifikke fortællinger, der forstærkes af et stemningsfuldt lyddesign. De litterære lydvandringer er tilgængelige i naturvejledernes app Naturlandet Sønderborg.</v>
+      </c>
+      <c r="M3" t="str">
+        <v>SPOR | Biblioteket Sønderborg</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://biblioteket.sonderborg.dk/spor</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://biblioteket.sonderborg.dk/spor#:~:text=vandring</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>